<commit_message>
add latest purchase date to divident file
</commit_message>
<xml_diff>
--- a/brokerQ2_股息入账汇总.xlsx
+++ b/brokerQ2_股息入账汇总.xlsx
@@ -524,7 +524,7 @@
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="11" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
-    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -728,7 +728,11 @@
         <f>"0800300405"</f>
         <v/>
       </c>
-      <c r="U2" s="7" t="n"/>
+      <c r="U2" s="7" t="inlineStr">
+        <is>
+          <t>不免</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
@@ -824,7 +828,11 @@
         <f>"0800300405"</f>
         <v/>
       </c>
-      <c r="U3" s="9" t="n"/>
+      <c r="U3" s="9" t="inlineStr">
+        <is>
+          <t>2019年5000股</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -921,7 +929,11 @@
           <t>B880865174</t>
         </is>
       </c>
-      <c r="U4" s="7" t="n"/>
+      <c r="U4" s="7" t="inlineStr">
+        <is>
+          <t>不免</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -1018,7 +1030,11 @@
           <t>B880865174</t>
         </is>
       </c>
-      <c r="U5" s="9" t="n"/>
+      <c r="U5" s="9" t="inlineStr">
+        <is>
+          <t>不免</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -1110,7 +1126,11 @@
         <f>"0800300405"</f>
         <v/>
       </c>
-      <c r="U6" s="7" t="n"/>
+      <c r="U6" s="7" t="inlineStr">
+        <is>
+          <t>2017年1000股</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -1206,7 +1226,11 @@
         <f>"0800300405"</f>
         <v/>
       </c>
-      <c r="U7" s="9" t="n"/>
+      <c r="U7" s="9" t="inlineStr">
+        <is>
+          <t>2025年9月</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U7"/>

</xml_diff>